<commit_message>
Feat: Ajustes generar ciclo de revision alexander martinez 2025-09-09
</commit_message>
<xml_diff>
--- a/src/assets/ejemplos/modelo/estructuraVisita.xlsx
+++ b/src/assets/ejemplos/modelo/estructuraVisita.xlsx
@@ -37,13 +37,13 @@
     <t xml:space="preserve">destinatario_direccion</t>
   </si>
   <si>
-    <t xml:space="preserve">ciudad</t>
-  </si>
-  <si>
     <t xml:space="preserve">destinatario_telefono</t>
   </si>
   <si>
     <t xml:space="preserve">destinatario_correo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unidades</t>
   </si>
   <si>
     <t xml:space="preserve">peso</t>
@@ -353,10 +353,9 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="40.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="12.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.39"/>
   </cols>
   <sheetData>
@@ -421,10 +420,10 @@
         <v>15</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="1" t="n">
         <v>3201457478</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>10</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
@@ -444,8 +443,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Página &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: unificar editar visita en rutear y agregar imprimir rótulo
- visita-editar-rutear ahora delega en VisitaFormularioComponent (15 campos completos)
- Antes solo tenía 10 campos; faltaban ciudad, correo, tiempo servicio, complemento, observación
- Agrega opción "Imprimir" al menú de tres puntos por fila en /rutear
- Plantilla Excel regenerada con 19 columnas (suma complemento, observacion, ciudad)
</commit_message>
<xml_diff>
--- a/src/assets/ejemplos/modelo/estructuraVisita.xlsx
+++ b/src/assets/ejemplos/modelo/estructuraVisita.xlsx
@@ -1,52 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -64,14 +44,82 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -396,103 +444,181 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>numero</v>
-      </c>
-      <c r="B1" t="str">
-        <v>fecha</v>
-      </c>
-      <c r="C1" t="str">
-        <v>documento</v>
-      </c>
-      <c r="D1" t="str">
-        <v>destinatario</v>
-      </c>
-      <c r="E1" t="str">
-        <v>destinatario_direccion</v>
-      </c>
-      <c r="F1" t="str">
-        <v>destinatario_telefono</v>
-      </c>
-      <c r="G1" t="str">
-        <v>destinatario_correo</v>
-      </c>
-      <c r="H1" t="str">
-        <v>unidades</v>
-      </c>
-      <c r="I1" t="str">
-        <v>peso</v>
-      </c>
-      <c r="J1" t="str">
-        <v>volumen</v>
-      </c>
-      <c r="K1" t="str">
-        <v>latitud</v>
-      </c>
-      <c r="L1" t="str">
-        <v>longitud</v>
-      </c>
-      <c r="M1" t="str">
-        <v>decodificado</v>
-      </c>
-      <c r="N1" t="str">
-        <v>tiempo_servicio</v>
-      </c>
-      <c r="O1" t="str">
-        <v>cita_inicio</v>
-      </c>
-      <c r="P1" t="str">
-        <v>cita_fin</v>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>numero</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>documento</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>destinatario</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>destinatario_direccion</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>destinatario_telefono</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>destinatario_correo</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>unidades</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>peso</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>volumen</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>latitud</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>longitud</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>decodificado</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>tiempo_servicio</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>cita_inicio</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>cita_fin</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>destinatario_direccion_complemento</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>observacion</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>ciudad</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" t="n">
         <v>123456</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>20241001</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>11111</v>
       </c>
-      <c r="D2" t="str">
-        <v>MARCO SANCHEZ</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Cra. 74 #No 48-37, Medellín, Antioquia</v>
-      </c>
-      <c r="F2">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MARCO SANCHEZ</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cra. 74 #No 48-37</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>3201457478</v>
       </c>
-      <c r="H2">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>cliente@correo.com</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
         <v>10</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="n">
         <v>1</v>
       </c>
-      <c r="J2">
+      <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="M2">
+      <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="N2">
+      <c r="N2" t="n">
         <v>3</v>
       </c>
-      <c r="O2" t="str">
-        <v>2024-10-01 08:00:00</v>
-      </c>
-      <c r="P2" t="str">
-        <v>2024-10-01 12:00:00</v>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2024-10-01 08:00:00</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2024-10-01 12:00:00</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Apto 301</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Entregar antes 12pm</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Medellin</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(visita): campo Recaudo en formulario manual y plantilla Excel
- visita-formulario.ts: control 'cobro' en el FormGroup, default 0, opcional.
- visita-formulario.html: input 'Recaudo' al lado de 'Tiempo servicio'.
- estructuraVisita.xlsx: agregada columna 'recaudo' (col T) con valor de
  ejemplo 50000.
- visita-detalle.html: la fila pasa de "Cobro" a "Recaudo" y formatea el
  valor como moneda COP.
</commit_message>
<xml_diff>
--- a/src/assets/ejemplos/modelo/estructuraVisita.xlsx
+++ b/src/assets/ejemplos/modelo/estructuraVisita.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,6 +548,11 @@
           <t>ciudad</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>recaudo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -616,6 +621,9 @@
         <is>
           <t>Medellin</t>
         </is>
+      </c>
+      <c r="T2" t="n">
+        <v>50000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(visita): campo Tarifa en formulario y plantilla Excel
- FormControl 'tarifa' con default 0 y min(0).
- Reset incluido en _defaultsFormulario.
- patchValue al editar trae el valor desde informacionVisita.tarifa.
- HTML modal: nuevo grid 2-cols con Tarifa y Recaudo, ambos con hint
  diferenciador ("precio del servicio" vs "contraentrega").
- HTML pagina completa: Tarifa al lado de Tiempo servicio y Recaudo.
- estructuraVisita.xlsx: columna U (21) "tarifa" con valor ejemplo 8500.
</commit_message>
<xml_diff>
--- a/src/assets/ejemplos/modelo/estructuraVisita.xlsx
+++ b/src/assets/ejemplos/modelo/estructuraVisita.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,6 +553,11 @@
           <t>recaudo</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>tarifa</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -624,6 +629,9 @@
       </c>
       <c r="T2" t="n">
         <v>50000</v>
+      </c>
+      <c r="U2" t="n">
+        <v>8500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>